<commit_message>
Add SH IQC Parks visits 13-14 (06/22 & 06/25) to master workbook
- Visit 13 (06/22, Parks, no batch): 36 inspected / 31 pass / 5 fail
- Visit 14 (06/25, Parks, no batch): 19 inspected / 16 pass / 3 fail

Both intact-only, PN normalized 668518->666518. Appended as visits 13-14 (processing
order, per the existing Visit 7/8 date-overlap convention); no SH->ATM rows since Parks
has no batch data. Updated metadata, raw rows, batch rollup (TOTAL now 772/719/53,
93.1% FPY), and notes 8 and 17. Edited at the XML level so the Defect Atlas photos and
all other sheets stay byte-for-byte identical.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
+++ b/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
@@ -6059,7 +6059,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.78"/>
@@ -6572,134 +6572,152 @@
         </is>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="18" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit 13</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-22</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rasmin Mujanovic</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Natalie</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit 14</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-25</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rasmin Mujanovic</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Natalie</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-    </row>
-    <row r="20" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B22" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C22" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D22" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E22" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F22" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G22" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H22" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="I20" s="11" t="s">
+      <c r="I22" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J22" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="K20" s="11" t="s">
+      <c r="K22" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="L20" s="11" t="s">
+      <c r="L22" s="11" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="H21" s="6" t="n">
-        <v>47</v>
-      </c>
-      <c r="I21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="15" t="n">
-        <f aca="false">IFERROR(H21/G21,0)</f>
-      </c>
-      <c r="K21" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="L21" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="H22" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="I22" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="J22" s="15" t="n">
-        <f aca="false">IFERROR(H22/G22,0)</f>
-      </c>
-      <c r="K22" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="L22" s="5" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6710,37 +6728,37 @@
         <v>53</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>3</v>
+        <v>47</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" s="15" t="n">
         <f aca="false">IFERROR(H23/G23,0)</f>
       </c>
       <c r="K23" s="16" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
         <v>104</v>
       </c>
@@ -6748,58 +6766,60 @@
         <v>53</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G24" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I24" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I24" s="6" t="n">
-        <v>0</v>
       </c>
       <c r="J24" s="15" t="n">
         <f aca="false">IFERROR(H24/G24,0)</f>
       </c>
-      <c r="K24" s="16"/>
+      <c r="K24" s="16" t="s">
+        <v>105</v>
+      </c>
       <c r="L24" s="5" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I25" s="6" t="n">
         <v>0</v>
@@ -6808,7 +6828,7 @@
         <f aca="false">IFERROR(H25/G25,0)</f>
       </c>
       <c r="K25" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>103</v>
@@ -6816,43 +6836,41 @@
     </row>
     <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>56</v>
+        <v>4</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" s="15" t="n">
         <f aca="false">IFERROR(H26/G26,0)</f>
       </c>
-      <c r="K26" s="16" t="s">
-        <v>111</v>
-      </c>
+      <c r="K26" s="16"/>
       <c r="L26" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
         <v>13</v>
       </c>
@@ -6860,31 +6878,31 @@
         <v>53</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J27" s="15" t="n">
         <f aca="false">IFERROR(H27/G27,0)</f>
       </c>
       <c r="K27" s="16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="L27" s="5" t="s">
         <v>103</v>
@@ -6898,31 +6916,31 @@
         <v>53</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J28" s="15" t="n">
         <f aca="false">IFERROR(H28/G28,0)</f>
       </c>
       <c r="K28" s="16" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="L28" s="5" t="s">
         <v>103</v>
@@ -6930,37 +6948,37 @@
     </row>
     <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29" s="15" t="n">
         <f aca="false">IFERROR(H29/G29,0)</f>
       </c>
       <c r="K29" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="L29" s="5" t="s">
         <v>103</v>
@@ -6968,37 +6986,37 @@
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J30" s="15" t="n">
         <f aca="false">IFERROR(H30/G30,0)</f>
       </c>
       <c r="K30" s="16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="L30" s="5" t="s">
         <v>103</v>
@@ -7012,31 +7030,31 @@
         <v>53</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J31" s="15" t="n">
         <f aca="false">IFERROR(H31/G31,0)</f>
       </c>
       <c r="K31" s="16" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="L31" s="5" t="s">
         <v>103</v>
@@ -7050,31 +7068,31 @@
         <v>53</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J32" s="15" t="n">
         <f aca="false">IFERROR(H32/G32,0)</f>
       </c>
       <c r="K32" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L32" s="5" t="s">
         <v>103</v>
@@ -7082,37 +7100,37 @@
     </row>
     <row r="33" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>118</v>
+        <v>14</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J33" s="15" t="n">
         <f aca="false">IFERROR(H33/G33,0)</f>
       </c>
       <c r="K33" s="16" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="L33" s="5" t="s">
         <v>103</v>
@@ -7120,43 +7138,43 @@
     </row>
     <row r="34" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J34" s="15" t="n">
         <f aca="false">IFERROR(H34/G34,0)</f>
       </c>
       <c r="K34" s="16" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="L34" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
         <v>118</v>
       </c>
@@ -7164,31 +7182,31 @@
         <v>53</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J35" s="15" t="n">
         <f aca="false">IFERROR(H35/G35,0)</f>
       </c>
       <c r="K35" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="L35" s="5" t="s">
         <v>103</v>
@@ -7202,31 +7220,31 @@
         <v>53</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H36" s="6" t="n">
         <v>29</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J36" s="15" t="n">
         <f aca="false">IFERROR(H36/G36,0)</f>
       </c>
       <c r="K36" s="16" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>103</v>
@@ -7234,89 +7252,89 @@
     </row>
     <row r="37" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>73</v>
+        <v>118</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J37" s="15" t="n">
         <f aca="false">IFERROR(H37/G37,0)</f>
       </c>
       <c r="K37" s="16" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="L37" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>16</v>
+        <v>120</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J38" s="15" t="n">
         <f aca="false">IFERROR(H38/G38,0)</f>
       </c>
       <c r="K38" s="16" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>128</v>
+        <v>73</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>53</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>58</v>
@@ -7328,58 +7346,60 @@
         <v>101</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="I39" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J39" s="15" t="n">
         <f aca="false">IFERROR(H39/G39,0)</f>
       </c>
-      <c r="K39" s="16"/>
+      <c r="K39" s="16" t="s">
+        <v>124</v>
+      </c>
       <c r="L39" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>129</v>
+        <v>16</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>100</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J40" s="15" t="n">
         <f aca="false">IFERROR(H40/G40,0)</f>
       </c>
       <c r="K40" s="16" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>103</v>
+        <v>127</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7390,22 +7410,22 @@
         <v>53</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I41" s="6" t="n">
         <v>0</v>
@@ -7426,52 +7446,54 @@
         <v>53</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J42" s="15" t="n">
         <f aca="false">IFERROR(H42/G42,0)</f>
       </c>
-      <c r="K42" s="16"/>
+      <c r="K42" s="16" t="s">
+        <v>130</v>
+      </c>
       <c r="L42" s="5" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>87</v>
+        <v>128</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
       <c r="G43" s="6" t="n">
         <v>7</v>
@@ -7487,121 +7509,85 @@
       </c>
       <c r="K43" s="16"/>
       <c r="L43" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-08</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martins</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5502428786</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">666541</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intact</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, intact</t>
-        </is>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>107</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="I44" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" s="15" t="n">
         <f aca="false">IFERROR(H44/G44,0)</f>
       </c>
-      <c r="K44" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 cut urethra</t>
-        </is>
-      </c>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Toni Cruz / Jesus</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-08</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martins</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5502428782</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">666506</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Non-intact</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, non-intact</t>
-        </is>
+      <c r="K44" s="16"/>
+      <c r="L44" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I45" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J45" s="15" t="n">
         <f aca="false">IFERROR(H45/G45,0)</f>
       </c>
-      <c r="K45" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 short block</t>
-        </is>
-      </c>
-      <c r="L45" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Toni Cruz / Jesus</t>
-        </is>
+      <c r="K45" s="16"/>
+      <c r="L45" s="5" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="46" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-15</t>
+          <t xml:space="preserve">2026-06-08</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -7611,7 +7597,7 @@
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">5502462845</t>
+          <t xml:space="preserve">5502428786</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -7630,10 +7616,10 @@
         </is>
       </c>
       <c r="G46" s="6" t="n">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="I46" s="6" t="n">
         <v>1</v>
@@ -7643,7 +7629,7 @@
       </c>
       <c r="K46" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 damaged bowel (source had two intact tally lines: 13/12/1 + 18/18/0, combined here)</t>
+          <t xml:space="preserve">1 cut urethra</t>
         </is>
       </c>
       <c r="L46" s="5" t="inlineStr">
@@ -7655,61 +7641,61 @@
     <row r="47" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-16</t>
+          <t xml:space="preserve">2026-06-08</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parks Family Meats</t>
+          <t xml:space="preserve">Martins</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">(no batch data)</t>
+          <t xml:space="preserve">5502428782</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">666518</t>
+          <t xml:space="preserve">666506</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Intact</t>
+          <t xml:space="preserve">Non-intact</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, intact, SM</t>
+          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, non-intact</t>
         </is>
       </c>
       <c r="G47" s="6" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="I47" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J47" s="15" t="n">
         <f aca="false">IFERROR(H47/G47,0)</f>
       </c>
       <c r="K47" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 bladder hole; 1 ureter damage (many blocks failed upstream from miscuts during removal — see notes)</t>
+          <t xml:space="preserve">1 short block</t>
         </is>
       </c>
       <c r="L47" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rasmin Mujanovic / Natalie</t>
+          <t xml:space="preserve">Toni Cruz / Jesus</t>
         </is>
       </c>
     </row>
     <row r="48" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-24</t>
+          <t xml:space="preserve">2026-06-15</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
@@ -7738,20 +7724,20 @@
         </is>
       </c>
       <c r="G48" s="6" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H48" s="6" t="n">
         <v>30</v>
       </c>
       <c r="I48" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J48" s="15" t="n">
         <f aca="false">IFERROR(H48/G48,0)</f>
       </c>
       <c r="K48" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 damaged bladder; 3 damaged membrane</t>
+          <t xml:space="preserve">1 damaged bowel (source had two intact tally lines: 13/12/1 + 18/18/0, combined here)</t>
         </is>
       </c>
       <c r="L48" s="5" t="inlineStr">
@@ -7760,170 +7746,270 @@
         </is>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3" t="s">
+    <row r="49" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-16</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, intact, SM</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="I49" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J49" s="15" t="n">
+        <f aca="false">IFERROR(H49/G49,0)</f>
+      </c>
+      <c r="K49" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 bladder hole; 1 ureter damage (many blocks failed upstream from miscuts during removal — see notes)</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rasmin Mujanovic / Natalie</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-24</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martins</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502462845</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666541</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, intact</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I50" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="J50" s="15" t="n">
+        <f aca="false">IFERROR(H50/G50,0)</f>
+      </c>
+      <c r="K50" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 damaged bladder; 3 damaged membrane</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Toni Cruz / Jesus</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-22</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, intact, SM</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="H51" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="I51" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J51" s="15" t="n">
+        <f aca="false">IFERROR(H51/G51,0)</f>
+      </c>
+      <c r="K51" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 bladder hole; 2 critical-area lacerations; 2 short blocks</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rasmin Mujanovic / Natalie</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-25</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tiss, porcine, fem, Pelvic block, intact, SM</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="H52" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="I52" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="15" t="n">
+        <f aca="false">IFERROR(H52/G52,0)</f>
+      </c>
+      <c r="K52" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 bladder hole; 1 ureter laceration; 1 short block</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rasmin Mujanovic / Natalie</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="3"/>
-      <c r="K50" s="3"/>
-      <c r="L50" s="3"/>
-    </row>
-    <row r="51" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="11" t="s">
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+    </row>
+    <row r="55" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B55" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C55" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D51" s="11" t="s">
+      <c r="D55" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E51" s="11" t="s">
+      <c r="E55" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="F51" s="11" t="s">
+      <c r="F55" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="G51" s="11" t="s">
+      <c r="G55" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="H51" s="11" t="s">
+      <c r="H55" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="I51" s="11" t="s">
+      <c r="I55" s="11" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B52" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D52" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F52" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="G52" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="H52" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I52" s="15" t="n">
-        <f aca="false">IFERROR(G52/F52,0)</f>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C53" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="D53" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="E53" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="F53" s="6" t="n">
-        <v>65</v>
-      </c>
-      <c r="G53" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="H53" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="I53" s="15" t="n">
-        <f aca="false">IFERROR(G53/F53,0)</f>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B54" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C54" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D54" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="E54" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="F54" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="G54" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="H54" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I54" s="15" t="n">
-        <f aca="false">IFERROR(G54/F54,0)</f>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B55" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C55" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="D55" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="E55" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="F55" s="6" t="n">
-        <v>57</v>
-      </c>
-      <c r="G55" s="6" t="n">
-        <v>56</v>
-      </c>
-      <c r="H55" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I55" s="15" t="n">
-        <f aca="false">IFERROR(G55/F55,0)</f>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B56" s="12" t="s">
         <v>59</v>
@@ -7935,16 +8021,16 @@
         <v>53</v>
       </c>
       <c r="E56" s="12" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="F56" s="6" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="G56" s="6" t="n">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I56" s="15" t="n">
         <f aca="false">IFERROR(G56/F56,0)</f>
@@ -7952,7 +8038,7 @@
     </row>
     <row r="57" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>66</v>
+        <v>56</v>
       </c>
       <c r="B57" s="12" t="s">
         <v>58</v>
@@ -7964,16 +8050,16 @@
         <v>53</v>
       </c>
       <c r="E57" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="F57" s="6" t="n">
         <v>65</v>
       </c>
-      <c r="F57" s="6" t="n">
-        <v>62</v>
-      </c>
       <c r="G57" s="6" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H57" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I57" s="15" t="n">
         <f aca="false">IFERROR(G57/F57,0)</f>
@@ -7981,7 +8067,7 @@
     </row>
     <row r="58" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B58" s="12" t="s">
         <v>59</v>
@@ -7993,16 +8079,16 @@
         <v>53</v>
       </c>
       <c r="E58" s="12" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="G58" s="6" t="n">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I58" s="15" t="n">
         <f aca="false">IFERROR(G58/F58,0)</f>
@@ -8010,7 +8096,7 @@
     </row>
     <row r="59" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B59" s="12" t="s">
         <v>58</v>
@@ -8022,16 +8108,16 @@
         <v>53</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="G59" s="6" t="n">
-        <v>87</v>
+        <v>56</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I59" s="15" t="n">
         <f aca="false">IFERROR(G59/F59,0)</f>
@@ -8039,28 +8125,28 @@
     </row>
     <row r="60" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D60" s="12" t="s">
         <v>53</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G60" s="6" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H60" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I60" s="15" t="n">
         <f aca="false">IFERROR(G60/F60,0)</f>
@@ -8068,28 +8154,28 @@
     </row>
     <row r="61" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="C61" s="12" t="s">
         <v>100</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="G61" s="6" t="n">
-        <v>11</v>
+        <v>58</v>
       </c>
       <c r="H61" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I61" s="15" t="n">
         <f aca="false">IFERROR(G61/F61,0)</f>
@@ -8097,25 +8183,25 @@
     </row>
     <row r="62" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D62" s="12" t="s">
         <v>53</v>
       </c>
       <c r="E62" s="12" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="F62" s="6" t="n">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="G62" s="6" t="n">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="H62" s="6" t="n">
         <v>2</v>
@@ -8126,28 +8212,28 @@
     </row>
     <row r="63" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D63" s="12" t="s">
         <v>53</v>
       </c>
       <c r="E63" s="12" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>36</v>
+        <v>93</v>
       </c>
       <c r="G63" s="6" t="n">
-        <v>36</v>
+        <v>87</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I63" s="15" t="n">
         <f aca="false">IFERROR(G63/F63,0)</f>
@@ -8155,198 +8241,158 @@
     </row>
     <row r="64" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="C64" s="12" t="s">
         <v>100</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="E64" s="12" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="F64" s="6" t="n">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="G64" s="6" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I64" s="15" t="n">
         <f aca="false">IFERROR(G64/F64,0)</f>
       </c>
     </row>
-    <row r="65" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="65" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E65" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H65" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I65" s="15" t="n">
+        <f aca="false">IFERROR(G65/F65,0)</f>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B66" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E66" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="G66" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="H66" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I66" s="15" t="n">
+        <f aca="false">IFERROR(G66/F66,0)</f>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B67" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E67" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="G67" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="H67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="15" t="n">
+        <f aca="false">IFERROR(G67/F67,0)</f>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E68" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="G68" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="H68" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="15" t="n">
+        <f aca="false">IFERROR(G68/F68,0)</f>
+      </c>
+    </row>
+    <row r="69" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">5502428786</t>
         </is>
       </c>
-      <c r="B65" s="12" t="inlineStr">
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">666541</t>
-        </is>
-      </c>
-      <c r="C65" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intact</t>
-        </is>
-      </c>
-      <c r="D65" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martins</t>
-        </is>
-      </c>
-      <c r="E65" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-08</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="G65" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="H65" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I65" s="15" t="n">
-        <f aca="false">IFERROR(G65/F65,0)</f>
-      </c>
-    </row>
-    <row r="66" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5502428782</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">666506</t>
-        </is>
-      </c>
-      <c r="C66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Non-intact</t>
-        </is>
-      </c>
-      <c r="D66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martins</t>
-        </is>
-      </c>
-      <c r="E66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-08</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="G66" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="H66" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I66" s="15" t="n">
-        <f aca="false">IFERROR(G66/F66,0)</f>
-      </c>
-    </row>
-    <row r="67" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5502462845</t>
-        </is>
-      </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">666541</t>
-        </is>
-      </c>
-      <c r="C67" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intact</t>
-        </is>
-      </c>
-      <c r="D67" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martins</t>
-        </is>
-      </c>
-      <c r="E67" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-15</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="n">
-        <v>31</v>
-      </c>
-      <c r="G67" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H67" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I67" s="15" t="n">
-        <f aca="false">IFERROR(G67/F67,0)</f>
-      </c>
-    </row>
-    <row r="68" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5502462845</t>
-        </is>
-      </c>
-      <c r="B68" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">666541</t>
-        </is>
-      </c>
-      <c r="C68" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Intact</t>
-        </is>
-      </c>
-      <c r="D68" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Martins</t>
-        </is>
-      </c>
-      <c r="E68" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-24</t>
-        </is>
-      </c>
-      <c r="F68" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="G68" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H68" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I68" s="15" t="n">
-        <f aca="false">IFERROR(G68/F68,0)</f>
-      </c>
-    </row>
-    <row r="69" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">(no batch data)</t>
-        </is>
-      </c>
-      <c r="B69" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">666518</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
@@ -8356,300 +8402,342 @@
       </c>
       <c r="D69" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Martins</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-08</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="G69" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I69" s="15" t="n">
+        <f aca="false">IFERROR(G69/F69,0)</f>
+      </c>
+    </row>
+    <row r="70" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502428782</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666506</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non-intact</t>
+        </is>
+      </c>
+      <c r="D70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martins</t>
+        </is>
+      </c>
+      <c r="E70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-08</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="G70" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I70" s="15" t="n">
+        <f aca="false">IFERROR(G70/F70,0)</f>
+      </c>
+    </row>
+    <row r="71" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502462845</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666541</t>
+        </is>
+      </c>
+      <c r="C71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="D71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martins</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-15</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="G71" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I71" s="15" t="n">
+        <f aca="false">IFERROR(G71/F71,0)</f>
+      </c>
+    </row>
+    <row r="72" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5502462845</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666541</t>
+        </is>
+      </c>
+      <c r="C72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="D72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Martins</t>
+        </is>
+      </c>
+      <c r="E72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-24</t>
+        </is>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="G72" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="H72" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I72" s="15" t="n">
+        <f aca="false">IFERROR(G72/F72,0)</f>
+      </c>
+    </row>
+    <row r="73" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="C73" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="D73" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Parks Family Meats</t>
         </is>
       </c>
-      <c r="E69" s="12" t="inlineStr">
+      <c r="E73" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-16</t>
         </is>
       </c>
-      <c r="F69" s="6" t="n">
+      <c r="F73" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="G69" s="6" t="n">
+      <c r="G73" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="H69" s="6" t="n">
+      <c r="H73" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="I69" s="15" t="n">
-        <f aca="false">IFERROR(G69/F69,0)</f>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="17" t="s">
+      <c r="I73" s="15" t="n">
+        <f aca="false">IFERROR(G73/F73,0)</f>
+      </c>
+    </row>
+    <row r="74" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="B74" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="C74" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="D74" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-22</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="G74" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="H74" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I74" s="15" t="n">
+        <f aca="false">IFERROR(G74/F74,0)</f>
+      </c>
+    </row>
+    <row r="75" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(no batch data)</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666518</t>
+        </is>
+      </c>
+      <c r="C75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Intact</t>
+        </is>
+      </c>
+      <c r="D75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parks Family Meats</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-06-25</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="G75" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H75" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I75" s="15" t="n">
+        <f aca="false">IFERROR(G75/F75,0)</f>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17"/>
-      <c r="E70" s="17"/>
-      <c r="F70" s="8" t="n">
-        <f aca="false">SUM(F52:F69)</f>
-      </c>
-      <c r="G70" s="8" t="n">
-        <f aca="false">SUM(G52:G69)</f>
-      </c>
-      <c r="H70" s="8" t="n">
-        <f aca="false">SUM(H52:H69)</f>
-      </c>
-      <c r="I70" s="9" t="n">
-        <f aca="false">IFERROR(G70/F70,0)</f>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="10" t="s">
+      <c r="B76" s="17"/>
+      <c r="C76" s="17"/>
+      <c r="D76" s="17"/>
+      <c r="E76" s="17"/>
+      <c r="F76" s="8" t="n">
+        <f aca="false">SUM(F56:F75)</f>
+      </c>
+      <c r="G76" s="8" t="n">
+        <f aca="false">SUM(G56:G75)</f>
+      </c>
+      <c r="H76" s="8" t="n">
+        <f aca="false">SUM(H56:H75)</f>
+      </c>
+      <c r="I76" s="9" t="n">
+        <f aca="false">IFERROR(G76/F76,0)</f>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B72" s="10"/>
-      <c r="C72" s="10"/>
-      <c r="D72" s="10"/>
-      <c r="E72" s="10"/>
-      <c r="F72" s="10"/>
-      <c r="G72" s="10"/>
-      <c r="H72" s="10"/>
-      <c r="I72" s="10"/>
-      <c r="J72" s="10"/>
-      <c r="K72" s="10"/>
-      <c r="L72" s="10"/>
-    </row>
-    <row r="73" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="11" t="s">
+      <c r="B78" s="10"/>
+      <c r="C78" s="10"/>
+      <c r="D78" s="10"/>
+      <c r="E78" s="10"/>
+      <c r="F78" s="10"/>
+      <c r="G78" s="10"/>
+      <c r="H78" s="10"/>
+      <c r="I78" s="10"/>
+      <c r="J78" s="10"/>
+      <c r="K78" s="10"/>
+      <c r="L78" s="10"/>
+    </row>
+    <row r="79" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="B73" s="11" t="s">
+      <c r="B79" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="C73" s="11" t="s">
+      <c r="C79" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="D73" s="11" t="s">
+      <c r="D79" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="E73" s="11" t="s">
+      <c r="E79" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="F73" s="11" t="s">
+      <c r="F79" s="11" t="s">
         <v>138</v>
       </c>
-      <c r="G73" s="11" t="s">
+      <c r="G79" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="H73" s="11" t="s">
+      <c r="H79" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="I73" s="11" t="s">
+      <c r="I79" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="J73" s="11" t="s">
+      <c r="J79" s="11" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B74" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C74" s="6" t="n">
-        <v>65</v>
-      </c>
-      <c r="D74" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="E74" s="15" t="n">
-        <f aca="false">IFERROR(D74/C74,0)</f>
-      </c>
-      <c r="F74" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A74)</f>
-      </c>
-      <c r="G74" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A74)</f>
-      </c>
-      <c r="H74" s="15" t="n">
-        <f aca="false">IFERROR(G74/F74,0)</f>
-      </c>
-      <c r="I74" s="6" t="n">
-        <f aca="false">D74-F74</f>
-      </c>
-      <c r="J74" s="16" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="B75" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C75" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="D75" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="E75" s="15" t="n">
-        <f aca="false">IFERROR(D75/C75,0)</f>
-      </c>
-      <c r="F75" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A75)</f>
-      </c>
-      <c r="G75" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A75)</f>
-      </c>
-      <c r="H75" s="15" t="n">
-        <f aca="false">IFERROR(G75/F75,0)</f>
-      </c>
-      <c r="I75" s="6" t="n">
-        <f aca="false">D75-F75</f>
-      </c>
-      <c r="J75" s="16" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B76" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C76" s="6" t="n">
-        <v>57</v>
-      </c>
-      <c r="D76" s="6" t="n">
-        <v>56</v>
-      </c>
-      <c r="E76" s="15" t="n">
-        <f aca="false">IFERROR(D76/C76,0)</f>
-      </c>
-      <c r="F76" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A76)</f>
-      </c>
-      <c r="G76" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A76)</f>
-      </c>
-      <c r="H76" s="15" t="n">
-        <f aca="false">IFERROR(G76/F76,0)</f>
-      </c>
-      <c r="I76" s="6" t="n">
-        <f aca="false">D76-F76</f>
-      </c>
-      <c r="J76" s="16" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="B77" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C77" s="6" t="n">
-        <v>52</v>
-      </c>
-      <c r="D77" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="E77" s="15" t="n">
-        <f aca="false">IFERROR(D77/C77,0)</f>
-      </c>
-      <c r="F77" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A77)</f>
-      </c>
-      <c r="G77" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A77)</f>
-      </c>
-      <c r="H77" s="15" t="n">
-        <f aca="false">IFERROR(G77/F77,0)</f>
-      </c>
-      <c r="I77" s="6" t="n">
-        <f aca="false">D77-F77</f>
-      </c>
-      <c r="J77" s="16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="B78" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="C78" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="D78" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="E78" s="15" t="n">
-        <f aca="false">IFERROR(D78/C78,0)</f>
-      </c>
-      <c r="F78" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A78)</f>
-      </c>
-      <c r="G78" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A78)</f>
-      </c>
-      <c r="H78" s="15" t="n">
-        <f aca="false">IFERROR(G78/F78,0)</f>
-      </c>
-      <c r="I78" s="6" t="n">
-        <f aca="false">D78-F78</f>
-      </c>
-      <c r="J78" s="16" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="B79" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C79" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="D79" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="E79" s="15" t="n">
-        <f aca="false">IFERROR(D79/C79,0)</f>
-      </c>
-      <c r="F79" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A79)</f>
-      </c>
-      <c r="G79" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A79)</f>
-      </c>
-      <c r="H79" s="15" t="n">
-        <f aca="false">IFERROR(G79/F79,0)</f>
-      </c>
-      <c r="I79" s="6" t="n">
-        <f aca="false">D79-F79</f>
-      </c>
-      <c r="J79" s="16" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="18" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="B80" s="18" t="s">
         <v>58</v>
       </c>
       <c r="C80" s="6" t="n">
-        <v>93</v>
+        <v>65</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="E80" s="15" t="n">
         <f aca="false">IFERROR(D80/C80,0)</f>
@@ -8667,21 +8755,21 @@
         <f aca="false">D80-F80</f>
       </c>
       <c r="J80" s="16" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="18" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B81" s="18" t="s">
         <v>59</v>
       </c>
       <c r="C81" s="6" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>71</v>
+        <v>7</v>
       </c>
       <c r="E81" s="15" t="n">
         <f aca="false">IFERROR(D81/C81,0)</f>
@@ -8699,21 +8787,21 @@
         <f aca="false">D81-F81</f>
       </c>
       <c r="J81" s="16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="18" t="s">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="B82" s="18" t="s">
         <v>58</v>
       </c>
       <c r="C82" s="6" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E82" s="15" t="n">
         <f aca="false">IFERROR(D82/C82,0)</f>
@@ -8731,21 +8819,21 @@
         <f aca="false">D82-F82</f>
       </c>
       <c r="J82" s="16" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="18" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="B83" s="18" t="s">
         <v>59</v>
       </c>
       <c r="C83" s="6" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E83" s="15" t="n">
         <f aca="false">IFERROR(D83/C83,0)</f>
@@ -8763,177 +8851,261 @@
         <f aca="false">D83-F83</f>
       </c>
       <c r="J83" s="16" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B84" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C84" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="D84" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="E84" s="15" t="n">
+        <f aca="false">IFERROR(D84/C84,0)</f>
+      </c>
+      <c r="F84" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A84)</f>
+      </c>
+      <c r="G84" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A84)</f>
+      </c>
+      <c r="H84" s="15" t="n">
+        <f aca="false">IFERROR(G84/F84,0)</f>
+      </c>
+      <c r="I84" s="6" t="n">
+        <f aca="false">D84-F84</f>
+      </c>
+      <c r="J84" s="16" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="B85" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C85" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="E85" s="15" t="n">
+        <f aca="false">IFERROR(D85/C85,0)</f>
+      </c>
+      <c r="F85" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A85)</f>
+      </c>
+      <c r="G85" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A85)</f>
+      </c>
+      <c r="H85" s="15" t="n">
+        <f aca="false">IFERROR(G85/F85,0)</f>
+      </c>
+      <c r="I85" s="6" t="n">
+        <f aca="false">D85-F85</f>
+      </c>
+      <c r="J85" s="16" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A86" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B86" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C86" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="D86" s="6" t="n">
+        <v>87</v>
+      </c>
+      <c r="E86" s="15" t="n">
+        <f aca="false">IFERROR(D86/C86,0)</f>
+      </c>
+      <c r="F86" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A86)</f>
+      </c>
+      <c r="G86" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A86)</f>
+      </c>
+      <c r="H86" s="15" t="n">
+        <f aca="false">IFERROR(G86/F86,0)</f>
+      </c>
+      <c r="I86" s="6" t="n">
+        <f aca="false">D86-F86</f>
+      </c>
+      <c r="J86" s="16" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A87" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B87" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C87" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="E87" s="15" t="n">
+        <f aca="false">IFERROR(D87/C87,0)</f>
+      </c>
+      <c r="F87" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A87)</f>
+      </c>
+      <c r="G87" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A87)</f>
+      </c>
+      <c r="H87" s="15" t="n">
+        <f aca="false">IFERROR(G87/F87,0)</f>
+      </c>
+      <c r="I87" s="6" t="n">
+        <f aca="false">D87-F87</f>
+      </c>
+      <c r="J87" s="16" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A88" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="B88" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="E88" s="15" t="n">
+        <f aca="false">IFERROR(D88/C88,0)</f>
+      </c>
+      <c r="F88" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A88)</f>
+      </c>
+      <c r="G88" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A88)</f>
+      </c>
+      <c r="H88" s="15" t="n">
+        <f aca="false">IFERROR(G88/F88,0)</f>
+      </c>
+      <c r="I88" s="6" t="n">
+        <f aca="false">D88-F88</f>
+      </c>
+      <c r="J88" s="16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A89" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="B89" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="E89" s="15" t="n">
+        <f aca="false">IFERROR(D89/C89,0)</f>
+      </c>
+      <c r="F89" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A89)</f>
+      </c>
+      <c r="G89" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A89)</f>
+      </c>
+      <c r="H89" s="15" t="n">
+        <f aca="false">IFERROR(G89/F89,0)</f>
+      </c>
+      <c r="I89" s="6" t="n">
+        <f aca="false">D89-F89</f>
+      </c>
+      <c r="J89" s="16" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="84" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="18" t="inlineStr">
+    <row r="90" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">5502462845</t>
         </is>
       </c>
-      <c r="B84" s="18" t="inlineStr">
+      <c r="B90" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">666541</t>
         </is>
       </c>
-      <c r="C84" s="6" t="n">
+      <c r="C90" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="D84" s="6" t="n">
+      <c r="D90" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="E84" s="15" t="n">
-        <f aca="false">IFERROR(D84/C84,0)</f>
-      </c>
-      <c r="F84" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A84)</f>
-      </c>
-      <c r="G84" s="6" t="n">
-        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A84)</f>
-      </c>
-      <c r="H84" s="15" t="n">
-        <f aca="false">IFERROR(G84/F84,0)</f>
-      </c>
-      <c r="I84" s="6" t="n">
-        <f aca="false">D84-F84</f>
-      </c>
-      <c r="J84" s="16" t="inlineStr">
+      <c r="E90" s="15" t="n">
+        <f aca="false">IFERROR(D90/C90,0)</f>
+      </c>
+      <c r="F90" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!F:F,'Receipt Summary'!E:E,A90)</f>
+      </c>
+      <c r="G90" s="6" t="n">
+        <f aca="false">SUMIFS('Receipt Summary'!G:G,'Receipt Summary'!E:E,A90)</f>
+      </c>
+      <c r="H90" s="15" t="n">
+        <f aca="false">IFERROR(G90/F90,0)</f>
+      </c>
+      <c r="I90" s="6" t="n">
+        <f aca="false">D90-F90</f>
+      </c>
+      <c r="J90" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">Newly harvested 06/15. SH sampled 31 intact, passed 30 (96.8%). Lot # reappears on the 06/24 tally (34 inspected / 30 passed) — recorded as a separate Visit 12, likely a tally-sheet lot carry-over (see notes). Not yet at ATM; expected in coming weeks.</t>
         </is>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="3" t="s">
+    <row r="92" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A92" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="3"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-    </row>
-    <row r="87" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="19" t="s">
-        <v>152</v>
-      </c>
-      <c r="B87" s="20" t="s">
-        <v>153</v>
-      </c>
-      <c r="C87" s="20"/>
-      <c r="D87" s="20"/>
-      <c r="E87" s="20"/>
-      <c r="F87" s="20"/>
-      <c r="G87" s="20"/>
-      <c r="H87" s="20"/>
-      <c r="I87" s="20"/>
-      <c r="J87" s="20"/>
-      <c r="K87" s="20"/>
-      <c r="L87" s="20"/>
-    </row>
-    <row r="88" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="B88" s="20" t="s">
-        <v>155</v>
-      </c>
-      <c r="C88" s="20"/>
-      <c r="D88" s="20"/>
-      <c r="E88" s="20"/>
-      <c r="F88" s="20"/>
-      <c r="G88" s="20"/>
-      <c r="H88" s="20"/>
-      <c r="I88" s="20"/>
-      <c r="J88" s="20"/>
-      <c r="K88" s="20"/>
-      <c r="L88" s="20"/>
-    </row>
-    <row r="89" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="B89" s="20" t="s">
-        <v>157</v>
-      </c>
-      <c r="C89" s="20"/>
-      <c r="D89" s="20"/>
-      <c r="E89" s="20"/>
-      <c r="F89" s="20"/>
-      <c r="G89" s="20"/>
-      <c r="H89" s="20"/>
-      <c r="I89" s="20"/>
-      <c r="J89" s="20"/>
-      <c r="K89" s="20"/>
-      <c r="L89" s="20"/>
-    </row>
-    <row r="90" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="B90" s="20" t="s">
-        <v>159</v>
-      </c>
-      <c r="C90" s="20"/>
-      <c r="D90" s="20"/>
-      <c r="E90" s="20"/>
-      <c r="F90" s="20"/>
-      <c r="G90" s="20"/>
-      <c r="H90" s="20"/>
-      <c r="I90" s="20"/>
-      <c r="J90" s="20"/>
-      <c r="K90" s="20"/>
-      <c r="L90" s="20"/>
-    </row>
-    <row r="91" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="B91" s="20" t="s">
-        <v>161</v>
-      </c>
-      <c r="C91" s="20"/>
-      <c r="D91" s="20"/>
-      <c r="E91" s="20"/>
-      <c r="F91" s="20"/>
-      <c r="G91" s="20"/>
-      <c r="H91" s="20"/>
-      <c r="I91" s="20"/>
-      <c r="J91" s="20"/>
-      <c r="K91" s="20"/>
-      <c r="L91" s="20"/>
-    </row>
-    <row r="92" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="B92" s="20" t="s">
-        <v>163</v>
-      </c>
-      <c r="C92" s="20"/>
-      <c r="D92" s="20"/>
-      <c r="E92" s="20"/>
-      <c r="F92" s="20"/>
-      <c r="G92" s="20"/>
-      <c r="H92" s="20"/>
-      <c r="I92" s="20"/>
-      <c r="J92" s="20"/>
-      <c r="K92" s="20"/>
-      <c r="L92" s="20"/>
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="H92" s="3"/>
+      <c r="I92" s="3"/>
+      <c r="J92" s="3"/>
+      <c r="K92" s="3"/>
+      <c r="L92" s="3"/>
     </row>
     <row r="93" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="19" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="B93" s="20" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="C93" s="20"/>
       <c r="D93" s="20"/>
@@ -8948,12 +9120,10 @@
     </row>
     <row r="94" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="B94" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Twelve inspection visits so far. Nine at Martins (Visits 1–5, 7, 9, 10, 12) and three at Parks (Visits 6, 8, 11). To extend, append new visit metadata, raw-data rows, and rollup rows; the TOTAL and SH→ATM sections then need refreshing.</t>
-        </is>
+        <v>154</v>
+      </c>
+      <c r="B94" s="20" t="s">
+        <v>155</v>
       </c>
       <c r="C94" s="20"/>
       <c r="D94" s="20"/>
@@ -8968,10 +9138,10 @@
     </row>
     <row r="95" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="19" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="B95" s="20" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="C95" s="20"/>
       <c r="D95" s="20"/>
@@ -8986,10 +9156,10 @@
     </row>
     <row r="96" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="19" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="B96" s="20" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C96" s="20"/>
       <c r="D96" s="20"/>
@@ -9004,10 +9174,10 @@
     </row>
     <row r="97" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="19" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="B97" s="20" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="C97" s="20"/>
       <c r="D97" s="20"/>
@@ -9022,10 +9192,10 @@
     </row>
     <row r="98" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="19" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B98" s="20" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="C98" s="20"/>
       <c r="D98" s="20"/>
@@ -9038,16 +9208,12 @@
       <c r="K98" s="20"/>
       <c r="L98" s="20"/>
     </row>
-    <row r="99" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13. New visits 9–12 (06/08–06/24)</t>
-        </is>
-      </c>
-      <c r="B99" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Visit 9 = 06/08 Martins; Visit 10 = 06/15 Martins; Visit 11 = 06/16 Parks (intact-only); Visit 12 = 06/24 Martins (intact-only). Source date/kill fields on several incoming sheets are volatile =NOW() captures (e.g. the Parks sheet sent 06/17 reads 06/16); the hand-entered harvest-date fields were used as the authoritative visit dates.</t>
-        </is>
+    <row r="99" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="B99" s="20" t="s">
+        <v>165</v>
       </c>
       <c r="C99" s="20"/>
       <c r="D99" s="20"/>
@@ -9060,15 +9226,13 @@
       <c r="K99" s="20"/>
       <c r="L99" s="20"/>
     </row>
-    <row r="100" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14. Lot-number carry-over recurs (Visits 9 &amp; 12)</t>
-        </is>
+    <row r="100" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="19" t="s">
+        <v>166</v>
       </c>
       <c r="B100" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Visit 9 (06/08) reuses Visit 7’s lots 5502428786/5502428782, and Visit 12 (06/24) reuses Visit 10’s intact lot 5502462845 — the same template carry-over pattern documented in note 9 for lot 5502421192. Each is recorded as its own visit with its own raw and rollup rows, but per the note-9 precedent only the FIRST occurrence of each lot is reconciled in the SH→ATM section, so the reused-lot inspections do not generate duplicate SH→ATM rows.</t>
+          <t xml:space="preserve">Fourteen inspection visits so far. Nine at Martins (Visits 1–5, 7, 9, 10, 12) and five at Parks (Visits 6, 8, 11, 13, 14). To extend, append new visit metadata, raw-data rows, and rollup rows; the TOTAL and SH→ATM sections then need refreshing.</t>
         </is>
       </c>
       <c r="C100" s="20"/>
@@ -9082,16 +9246,12 @@
       <c r="K100" s="20"/>
       <c r="L100" s="20"/>
     </row>
-    <row r="101" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15. Visit 10 (06/15) — two intact tally lines combined; no non-intact</t>
-        </is>
-      </c>
-      <c r="B101" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The source recorded two intact 666541 lines on 06/15 (13/12/1 and 18/18/0); they share date, lot and condition, so they are combined into a single raw row (31/30/1). No non-intact units were collected (the SH had met its non-intact quota and run low on labels), so lot 5502462842 appears in the metadata but has no raw/rollup row.</t>
-        </is>
+    <row r="101" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="B101" s="20" t="s">
+        <v>169</v>
       </c>
       <c r="C101" s="20"/>
       <c r="D101" s="20"/>
@@ -9104,16 +9264,12 @@
       <c r="K101" s="20"/>
       <c r="L101" s="20"/>
     </row>
-    <row r="102" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16. Visit 11 (06/16 Parks) — heavy upstream miscut losses</t>
-        </is>
-      </c>
-      <c r="B102" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The inspector noted ~100 pigs slaughtered, with the majority of blocks failing BEFORE reaching IQC due to miscuts during block removal. Of the 16 that reached inspection, 14 passed (1 bladder hole, 1 ureter damage). That upstream loss is a Parks harvest-technique signal not captured in the pass/fail counts here. PN normalized 668518 → 666518 per note 10. Separately, the “PARKS0603” sheet (internal date 06/02, 7/7 intact, no batch) is the SAME inspection already recorded as Visit 8 and was not re-added.</t>
-        </is>
+    <row r="102" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="B102" s="20" t="s">
+        <v>171</v>
       </c>
       <c r="C102" s="20"/>
       <c r="D102" s="20"/>
@@ -9126,21 +9282,171 @@
       <c r="K102" s="20"/>
       <c r="L102" s="20"/>
     </row>
+    <row r="103" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="B103" s="20" t="s">
+        <v>173</v>
+      </c>
+      <c r="C103" s="20"/>
+      <c r="D103" s="20"/>
+      <c r="E103" s="20"/>
+      <c r="F103" s="20"/>
+      <c r="G103" s="20"/>
+      <c r="H103" s="20"/>
+      <c r="I103" s="20"/>
+      <c r="J103" s="20"/>
+      <c r="K103" s="20"/>
+      <c r="L103" s="20"/>
+    </row>
+    <row r="104" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A104" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="B104" s="20" t="s">
+        <v>175</v>
+      </c>
+      <c r="C104" s="20"/>
+      <c r="D104" s="20"/>
+      <c r="E104" s="20"/>
+      <c r="F104" s="20"/>
+      <c r="G104" s="20"/>
+      <c r="H104" s="20"/>
+      <c r="I104" s="20"/>
+      <c r="J104" s="20"/>
+      <c r="K104" s="20"/>
+      <c r="L104" s="20"/>
+    </row>
+    <row r="105" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13. New visits 9–12 (06/08–06/24)</t>
+        </is>
+      </c>
+      <c r="B105" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit 9 = 06/08 Martins; Visit 10 = 06/15 Martins; Visit 11 = 06/16 Parks (intact-only); Visit 12 = 06/24 Martins (intact-only). Source date/kill fields on several incoming sheets are volatile =NOW() captures (e.g. the Parks sheet sent 06/17 reads 06/16); the hand-entered harvest-date fields were used as the authoritative visit dates.</t>
+        </is>
+      </c>
+      <c r="C105" s="20"/>
+      <c r="D105" s="20"/>
+      <c r="E105" s="20"/>
+      <c r="F105" s="20"/>
+      <c r="G105" s="20"/>
+      <c r="H105" s="20"/>
+      <c r="I105" s="20"/>
+      <c r="J105" s="20"/>
+      <c r="K105" s="20"/>
+      <c r="L105" s="20"/>
+    </row>
+    <row r="106" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14. Lot-number carry-over recurs (Visits 9 &amp; 12)</t>
+        </is>
+      </c>
+      <c r="B106" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Visit 9 (06/08) reuses Visit 7’s lots 5502428786/5502428782, and Visit 12 (06/24) reuses Visit 10’s intact lot 5502462845 — the same template carry-over pattern documented in note 9 for lot 5502421192. Each is recorded as its own visit with its own raw and rollup rows, but per the note-9 precedent only the FIRST occurrence of each lot is reconciled in the SH→ATM section, so the reused-lot inspections do not generate duplicate SH→ATM rows.</t>
+        </is>
+      </c>
+      <c r="C106" s="20"/>
+      <c r="D106" s="20"/>
+      <c r="E106" s="20"/>
+      <c r="F106" s="20"/>
+      <c r="G106" s="20"/>
+      <c r="H106" s="20"/>
+      <c r="I106" s="20"/>
+      <c r="J106" s="20"/>
+      <c r="K106" s="20"/>
+      <c r="L106" s="20"/>
+    </row>
+    <row r="107" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15. Visit 10 (06/15) — two intact tally lines combined; no non-intact</t>
+        </is>
+      </c>
+      <c r="B107" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The source recorded two intact 666541 lines on 06/15 (13/12/1 and 18/18/0); they share date, lot and condition, so they are combined into a single raw row (31/30/1). No non-intact units were collected (the SH had met its non-intact quota and run low on labels), so lot 5502462842 appears in the metadata but has no raw/rollup row.</t>
+        </is>
+      </c>
+      <c r="C107" s="20"/>
+      <c r="D107" s="20"/>
+      <c r="E107" s="20"/>
+      <c r="F107" s="20"/>
+      <c r="G107" s="20"/>
+      <c r="H107" s="20"/>
+      <c r="I107" s="20"/>
+      <c r="J107" s="20"/>
+      <c r="K107" s="20"/>
+      <c r="L107" s="20"/>
+    </row>
+    <row r="108" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">16. Visit 11 (06/16 Parks) — heavy upstream miscut losses</t>
+        </is>
+      </c>
+      <c r="B108" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The inspector noted ~100 pigs slaughtered, with the majority of blocks failing BEFORE reaching IQC due to miscuts during block removal. Of the 16 that reached inspection, 14 passed (1 bladder hole, 1 ureter damage). That upstream loss is a Parks harvest-technique signal not captured in the pass/fail counts here. PN normalized 668518 → 666518 per note 10. Separately, the “PARKS0603” sheet (internal date 06/02, 7/7 intact, no batch) is the SAME inspection already recorded as Visit 8 and was not re-added.</t>
+        </is>
+      </c>
+      <c r="C108" s="20"/>
+      <c r="D108" s="20"/>
+      <c r="E108" s="20"/>
+      <c r="F108" s="20"/>
+      <c r="G108" s="20"/>
+      <c r="H108" s="20"/>
+      <c r="I108" s="20"/>
+      <c r="J108" s="20"/>
+      <c r="K108" s="20"/>
+      <c r="L108" s="20"/>
+    </row>
+    <row r="109" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">17. New Parks visits 13 (06/22) &amp; 14 (06/25)</t>
+        </is>
+      </c>
+      <c r="B109" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Two more intact-only Parks inspections (no batch data; PN normalized 668518 → 666518). Visit 13 (06/22) = 36 inspected / 31 pass / 5 fail (1 bladder hole, 2 critical-area lacerations, 2 short blocks); Visit 14 (06/25) = 19 inspected / 16 pass / 3 fail (1 bladder hole, 1 ureter laceration, 1 short block). Both were received after Visit 12, so Visit 13’s harvest date (06/22) precedes Visit 12’s (06/24 Martins) — visit numbers reflect processing order, as with the existing Visit 7/8 overlap. No batch on either, so neither has an SH→ATM link (consistent with Visits 6, 8 and 11). Short blocks and critical-zone mesentery damage continue to dominate Parks scrap.</t>
+        </is>
+      </c>
+      <c r="C109" s="20"/>
+      <c r="D109" s="20"/>
+      <c r="E109" s="20"/>
+      <c r="F109" s="20"/>
+      <c r="G109" s="20"/>
+      <c r="H109" s="20"/>
+      <c r="I109" s="20"/>
+      <c r="J109" s="20"/>
+      <c r="K109" s="20"/>
+      <c r="L109" s="20"/>
+      <c r="C109" s="20"/>
+      <c r="D109" s="20"/>
+      <c r="E109" s="20"/>
+      <c r="F109" s="20"/>
+      <c r="G109" s="20"/>
+      <c r="H109" s="20"/>
+      <c r="I109" s="20"/>
+      <c r="J109" s="20"/>
+      <c r="K109" s="20"/>
+      <c r="L109" s="20"/>
+    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A4:L4"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A50:L50"/>
-    <mergeCell ref="A72:L72"/>
-    <mergeCell ref="A86:L86"/>
-    <mergeCell ref="B87:L87"/>
-    <mergeCell ref="B88:L88"/>
-    <mergeCell ref="B89:L89"/>
-    <mergeCell ref="B90:L90"/>
-    <mergeCell ref="B91:L91"/>
-    <mergeCell ref="B92:L92"/>
+    <mergeCell ref="A21:L21"/>
+    <mergeCell ref="A54:L54"/>
+    <mergeCell ref="A78:L78"/>
+    <mergeCell ref="A92:L92"/>
     <mergeCell ref="B93:L93"/>
     <mergeCell ref="B94:L94"/>
     <mergeCell ref="B95:L95"/>
@@ -9151,6 +9457,13 @@
     <mergeCell ref="B100:L100"/>
     <mergeCell ref="B101:L101"/>
     <mergeCell ref="B102:L102"/>
+    <mergeCell ref="B103:L103"/>
+    <mergeCell ref="B104:L104"/>
+    <mergeCell ref="B105:L105"/>
+    <mergeCell ref="B106:L106"/>
+    <mergeCell ref="B107:L107"/>
+    <mergeCell ref="B108:L108"/>
+    <mergeCell ref="B109:L109"/>
   </mergeCells>
   <conditionalFormatting sqref="J17:J39">
     <cfRule type="colorScale" priority="2">

</xml_diff>

<commit_message>
Add SmartAssessment sheet with root-cause analysis notes
New worksheet capturing Claude's working assessment: objective (upstream
root-causing to improve harvesting first-pass yield at Parks & Martins), the
stage/yield pipeline model and the unmeasured harvesting-loss gap, the Parks
05/11 critical-mesentery event as a root-cause success story, defect-origin
tagging (harvesting vs freeze/thaw vs spec-drift), the SH-floor vs ATM yield
gap, the 666541/666506 spec correction (supersedes the earlier downgrade
assumption), data-quality caveats, and recommended next steps.

Added as a new worksheet at the XML level so the Defect Atlas photos and all
other sheets remain byte-for-byte identical.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
+++ b/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
@@ -10,6 +10,7 @@
   <sheets>
     <sheet name="Defect Trends- ATM" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Slaughterhouse IQC" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="SmartAssessment" sheetId="12" state="visible" r:id="rId15"/>
     <sheet name="Receipt Summary" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Master Data" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Defect Pivot 666541-F" sheetId="5" state="visible" r:id="rId7"/>
@@ -6054,6 +6055,263 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A37"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="98" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SmartAssessment — Pelvic Block Quality (Claude analysis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Author: Claude · Compiled 2026-06-26 · Scope: Slaughterhouse IQC visits 1–14 + ATM receipt data. These are working analyst notes and interpretation — verify with Quality before any external/supplier use.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. OBJECTIVE (as understood)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Root-cause pelvic-block defects to their point of origin UPSTREAM — before the harvesting tech consolidates the pelvic block, and ideally back to slaughter/evisceration (handling of the main tissue block and GI). Goal: raise HARVESTING FIRST-PASS YIELD = successful pelvic blocks consolidated ÷ main tissue blocks the harvesting tech receives. Active at BOTH suppliers: Parks (already engaged) and Martins (sampling defective pelvics and bringing them to ATM for evaluation/root-cause). This is a yield-improvement / root-cause program, not a supplier down-select.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. THE QUALITY PIPELINE — WHERE YIELD IS LOST</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage model</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stage 0  Upstream: slaughter + evisceration; handling of the main tissue block / GI.
+Stage 1  Harvesting: SH tech consolidates the pelvic block  ← first major yield loss, today largely UNMEASURED.
+Stage 2  SH-floor IQC: our ATM inspector, PRE-freeze — this is the current '# Inspected / Pass / Fail'.
+Stage 3  Freeze.
+Stage 4  ATM receipt: POST-freeze — the gate tied to performance goals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Key gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The tally sheets only count blocks that REACH our SH inspector. Blocks lost during harvesting (miscuts before presentation) are NOT in the pass/fail counts. See Parks Visit 11 (06/16): '~100 pigs slaughtered, the majority of blocks failed BEFORE reaching IQC due to miscuts during block removal.' That upstream loss IS the harvesting first-pass yield this program targets — and it is currently invisible. RECOMMEND adding two fields to the tally template: (a) main blocks received by harvesting tech, (b) blocks rejected at harvesting before IQC. Then harvesting FPY can be computed instead of inferred from a note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. PARKS 05/11 CRITICAL-MESENTERY EVENT — ROOT-CAUSE SUCCESS STORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATM receipt 05/11 (PN 666518): 220 received, 195 scrapped (88.6% rejection), of which 187 were critical mesentery holes/lacerations. This ONE event is 187 of Parks's 218 total critical-mesentery defects across the entire record — it dominates the Parks picture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed REAL (per Quality). Root cause: a harvesting cut that was dividing the mesentery from the block, plus bowel-area handling issues the slaughterhouse was unaware of. Corrected via training + monitoring; monthly verification calls ongoing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Post-intervention SH-floor visits (05/28 → 06/25) show NO recurrence of catastrophic rejection — yields 69–100%, steady ~84–88% recently. Residual scrap is now dominated by 'short blocks' and 'critical-area lacerations.' Read: the program fixed the catastrophic failure mode; a residual mesentery-length / critical-zone signal remains and is the next root-cause target at Parks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. WHERE DEFECTS ORIGINATE (origin tagging for root-cause)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Upstream / harvesting (the target of this program): critical mesentery hole/laceration; the mesentery-dividing cut; mesentery length too short (≤7" / 'short block'); bowel, bladder and urethra lacerations from miscuts; blood clots.
+• Freeze/thaw-attributable (per Quality — appear POST-thaw at ATM, not at the SH floor): small lacerations. These should NOT be charged to the harvesting tech's FPY; they explain part of the SH→ATM gap.
+• Spec / measurement drift (already in the IQC notes): bladder-length lower spec changed &lt;3"→&lt;2"; 'mesentery ≤7"' first measured 03/30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Recommendation</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">When ATM root-cause data arrives, tag each scrapped unit as harvesting-origin vs freeze/thaw-origin vs spec-drift, so the harvesting-FPY metric is not polluted by freeze/thaw damage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5. SH-FLOOR vs ATM YIELD (the stage gap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH-floor pass (pre-freeze): Martins 94.4% (640/678), Parks 84.0% (79/94).
+ATM receipt (post-freeze, rolling): Martins ~85.4% accepted (2119/2481), Parks ~39.8% (167/420) — Parks dominated by the 05/11 event.
+The SH→ATM gap is partly REAL freeze/thaw damage (small lacerations) and partly that ATM is a stricter/later gate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caveat</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only 3 lots currently have BOTH SH and ATM data (5502378434, 5502391862, 5502404928). The cleanest freeze/thaw proxy is the SH-pass → ATM-accept delta on MATCHED lots; we need more matched lots — especially post-intervention Parks — before trusting the gap quantitatively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6. 666541 vs 666506 — SPEC CORRECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Per Quality (06/26): 666506 = pelvic block with the MORE stringent spec; 666541 = the same part, LESS strict, and tied to ATM performance goals — so protecting 666541's ATM yield is the priority metric.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ Supersedes earlier assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This REVERSES the workbook's earlier framing (Slaughterhouse IQC note 1 / README) that treated 666506 as a 'downgrade/recovery' grade. Naming tension to reconcile: the tally sheets label 666541 'intact' and 666506 'non intact,' and some scrap notes say defective units were 'moved to non-intact' — wording that reads like a downgrade, which is hard to square with 666506 being the TIGHTER spec. Worth a one-line confirmation so labels and spec hierarchy agree. (I have NOT edited the old notes — flagging only.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7. DATA-QUALITY CAVEATS AFFECTING THIS ASSESSMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Parks SH sample is small (94 units, 5 visits) — supplier comparisons are directional, not statistical.
+• ATM Parks data currently ends 05/11, which PRE-DATES the SH-floor inspections (start 05/28) — so there is no clean post-intervention stage-to-stage comparison for Parks yet.
+• Lot-number carry-overs (Visits 5, 9, 12) mean some 'lots' repeat across weeks — see IQC notes 9 &amp; 14.
+• Several incoming tally dates are volatile =NOW() captures; hand-entered harvest dates were used as authoritative.
+• ATM data will soon lose batch numbers (Tableau) — a separate batch-less sheet is planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8. RECOMMENDED NEXT STEPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Add harvesting-FPY capture to the tally template (main blocks received; blocks rejected pre-IQC) so upstream loss is measured, not inferred.
+2. Tag ATM scrap by stage-of-origin (harvesting vs freeze/thaw vs spec-drift); keep freeze/thaw small-lacerations out of the harvesting-FPY denominator.
+3. Build a matched-lot SH→ATM tracker as more lots gain both stages — prioritize post-intervention Parks lots to verify the 05/11 fix holds through freeze/thaw.
+4. Reconcile the 666506 / 'non-intact' naming vs the tighter-spec definition; once confirmed, update IQC note 1 and the README.
+5. Continue monthly supplier calls; trend the residual Parks 'short block' / critical-zone signal and the Martins sampled-defect root-causes.
+6. When Tableau ATM data lands, link defect categories to stage-of-origin in the new batch-less sheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
Fix Slaughterhouse IQC formatting: CF ranges, row heights, freeze panes
- Re-point the four color-scale ranges that my earlier row inserts left stranded
  at pre-insert coordinates. The rollup-yield scale had drifted onto the # Fail
  count column (showing 0 fails as red, 1-2 as green); scales now sit on the
  actual yield columns: J23:J52, I56:I75, E80:E90, H80:H90.
- Set explicit row heights on all added rows (metadata, raw, rollup, SH->ATM,
  notes) to match each section and fully show wrapped scrap reasons / notes.
- Lighten freeze panes from 20 frozen rows to just the title row so the stacked
  tables scroll naturally.

XML-level edit; Defect Atlas photos and all other sheets unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
+++ b/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
@@ -6642,7 +6642,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A14" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Visit 9</t>
@@ -6689,7 +6689,7 @@
         </is>
       </c>
     </row>
-    <row r="15" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A15" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Visit 10</t>
@@ -6736,7 +6736,7 @@
         </is>
       </c>
     </row>
-    <row r="16" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A16" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Visit 11</t>
@@ -6783,7 +6783,7 @@
         </is>
       </c>
     </row>
-    <row r="17" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A17" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Visit 12</t>
@@ -6830,7 +6830,7 @@
         </is>
       </c>
     </row>
-    <row r="18" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A18" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Visit 13</t>
@@ -6877,7 +6877,7 @@
         </is>
       </c>
     </row>
-    <row r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A19" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">Visit 14</t>
@@ -7842,7 +7842,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="46" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A46" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-08</t>
@@ -7896,7 +7896,7 @@
         </is>
       </c>
     </row>
-    <row r="47" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A47" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-08</t>
@@ -7950,7 +7950,7 @@
         </is>
       </c>
     </row>
-    <row r="48" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="27.0" customHeight="true">
       <c r="A48" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-15</t>
@@ -8004,7 +8004,7 @@
         </is>
       </c>
     </row>
-    <row r="49" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="40.5" customHeight="true">
       <c r="A49" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-16</t>
@@ -8058,7 +8058,7 @@
         </is>
       </c>
     </row>
-    <row r="50" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A50" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-24</t>
@@ -8112,7 +8112,7 @@
         </is>
       </c>
     </row>
-    <row r="51" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="27.0" customHeight="true">
       <c r="A51" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-22</t>
@@ -8166,7 +8166,7 @@
         </is>
       </c>
     </row>
-    <row r="52" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="27.0" customHeight="true">
       <c r="A52" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-06-25</t>
@@ -8642,7 +8642,7 @@
         <f aca="false">IFERROR(G68/F68,0)</f>
       </c>
     </row>
-    <row r="69" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A69" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">5502428786</t>
@@ -8681,7 +8681,7 @@
         <f aca="false">IFERROR(G69/F69,0)</f>
       </c>
     </row>
-    <row r="70" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A70" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">5502428782</t>
@@ -8720,7 +8720,7 @@
         <f aca="false">IFERROR(G70/F70,0)</f>
       </c>
     </row>
-    <row r="71" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A71" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">5502462845</t>
@@ -8759,7 +8759,7 @@
         <f aca="false">IFERROR(G71/F71,0)</f>
       </c>
     </row>
-    <row r="72" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A72" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">5502462845</t>
@@ -8798,7 +8798,7 @@
         <f aca="false">IFERROR(G72/F72,0)</f>
       </c>
     </row>
-    <row r="73" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A73" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">(no batch data)</t>
@@ -8837,7 +8837,7 @@
         <f aca="false">IFERROR(G73/F73,0)</f>
       </c>
     </row>
-    <row r="74" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A74" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">(no batch data)</t>
@@ -8876,7 +8876,7 @@
         <f aca="false">IFERROR(G74/F74,0)</f>
       </c>
     </row>
-    <row r="75" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="13.5" customHeight="true">
       <c r="A75" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">(no batch data)</t>
@@ -9304,7 +9304,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="90" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="72.0" customHeight="true">
       <c r="A90" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">5502462845</t>
@@ -9576,7 +9576,7 @@
       <c r="K104" s="20"/>
       <c r="L104" s="20"/>
     </row>
-    <row r="105" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="48.0" customHeight="true">
       <c r="A105" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">13. New visits 9–12 (06/08–06/24)</t>
@@ -9598,7 +9598,7 @@
       <c r="K105" s="20"/>
       <c r="L105" s="20"/>
     </row>
-    <row r="106" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="48.0" customHeight="true">
       <c r="A106" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">14. Lot-number carry-over recurs (Visits 9 &amp; 12)</t>
@@ -9620,7 +9620,7 @@
       <c r="K106" s="20"/>
       <c r="L106" s="20"/>
     </row>
-    <row r="107" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="48.0" customHeight="true">
       <c r="A107" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">15. Visit 10 (06/15) — two intact tally lines combined; no non-intact</t>
@@ -9642,7 +9642,7 @@
       <c r="K107" s="20"/>
       <c r="L107" s="20"/>
     </row>
-    <row r="108" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="48.0" customHeight="true">
       <c r="A108" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">16. Visit 11 (06/16 Parks) — heavy upstream miscut losses</t>
@@ -9664,7 +9664,7 @@
       <c r="K108" s="20"/>
       <c r="L108" s="20"/>
     </row>
-    <row r="109" customFormat="false" hidden="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" hidden="false" outlineLevel="0" collapsed="false" ht="48.0" customHeight="true">
       <c r="A109" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">17. New Parks visits 13 (06/22) &amp; 14 (06/25)</t>
@@ -9723,7 +9723,7 @@
     <mergeCell ref="B108:L108"/>
     <mergeCell ref="B109:L109"/>
   </mergeCells>
-  <conditionalFormatting sqref="J17:J39">
+  <conditionalFormatting sqref="J23:J52">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -9735,7 +9735,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I43:I55">
+  <conditionalFormatting sqref="I56:I75">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -9747,7 +9747,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E60:E69">
+  <conditionalFormatting sqref="E80:E90">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0.7"/>
@@ -9759,7 +9759,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H60:H69">
+  <conditionalFormatting sqref="H80:H90">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0.7"/>

</xml_diff>

<commit_message>
Add ATM_Scrap_TableuData tab summarizing June Tableau scrap data
New batch-less ATM (post-freeze/thaw) tab summarizing the two June Tableau
charts for Martins parts 666541 & 666506:
- Weekly scrap % trend (5/25-6/29) with a red/yellow/green heatmap vs the 5% goal
- Overall scrap % by part (666541 4.6%, 666506 0.4%)
- Stage-to-stage lag correlation (ATM week <- SH harvest ~4-6 weeks prior) using
  the Martins SH 666541 scrap from the Slaughterhouse IQC tab
- Key takeaways + notes/assumptions (line->part mapping, lag band, no lot linkage)

Original Tableau screenshots not embedded (image files unavailable). Added as a
new worksheet at the XML level so the Defect Atlas photos and all other sheets
remain byte-for-byte identical.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
+++ b/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Defect Trends- ATM" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Slaughterhouse IQC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="SmartAssessment" sheetId="12" state="visible" r:id="rId15"/>
+    <sheet name="ATM_Scrap_TableuData" sheetId="13" state="visible" r:id="rId16"/>
     <sheet name="Receipt Summary" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Master Data" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Defect Pivot 666541-F" sheetId="5" state="visible" r:id="rId7"/>
@@ -6312,6 +6313,473 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F36"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="true">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATM Scrap — Tableau Data (post-freeze / thaw)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="true">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source: Tableau “Top 5 Part” scrap views, June 2026. ATM = receipt inspection AFTER freeze/thaw (product sits frozen ~1–1.5 months), so this month reflects SH harvest from roughly late-April to late-May. No batch/lot numbers in the ATM feed, so cross-stage links are by time-window + part only. Values read from the two charts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="18" customHeight="true">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WEEKLY SCRAP % TREND — JUNE 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Week (ATM receipt)</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666541 Scrap %</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666506 Scrap %</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Goal</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5/25</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/1</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/8</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/15</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/22</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/29</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13" ht="18" customHeight="true">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OVERALL SCRAP % BY PART — JUNE 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Part</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">June Scrap %</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vs 5% Goal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666541</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DV Tech Pelvic Block (F), intact — performance-goal part</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under (0.4 pt below goal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">666506</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pelvic Block, non-intact — tighter spec</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Under</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18" ht="18" customHeight="true">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGE-TO-STAGE LAG CORRELATION  (ATM week  ←  SH harvest ~4–6 weeks earlier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="true">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Directional only: ATM is weekly, SH visits are sporadic, and there is no lot linkage. SH 666541 scrap below is from the Martins intact rows on the Slaughterhouse IQC tab for the matching harvest window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATM week</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATM 666541 scrap</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH harvest window</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SH 666541 scrap (Martins)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5/25</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~4/13–4/22</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4.9% blended — 4/15 visit spiked to 23.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/1</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="n">
+        <v>0.063</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~4/20–4/29</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.8% (4/22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/8</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="n">
+        <v>0.074</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~4/27–5/6</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.5% (5/4 + 5/6; 5/6 = 12.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/15</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~5/4–5/13</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.5% (5/6 = 12.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/22</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="n">
+        <v>0.032</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~5/11–5/20</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.5% (5/18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6/29</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">~5/18–5/27</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.8% (5/18–5/27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28" ht="18" customHeight="true">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KEY TAKEAWAYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="true">
+      <c r="A29" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• 666541 (the performance-goal part) fell 25% → 0% across June and finished the month at 4.6% overall — just under the 5% goal. One early spike (25% on the 5/25 receipt) drove most of the month; it is the part to watch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="true">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• 666506 (tighter spec) held ~0% all month (0.4% overall) — well controlled through freeze/thaw.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="true">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Lag alignment: the 25% ATM spike (5/25) lands ~5–6 weeks after the roughest SH visit (4/15, 23.5% scrap) — consistent with the ~1–1.5-month freeze dwell and with defects originating upstream at harvest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="true">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Both parts trend down into summer, matching the harvesting-training improvements at the slaughterhouses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34" ht="18" customHeight="true">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NOTES &amp; ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="56" customHeight="true">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line→part mapping (dark = 666541, light = 666506) inferred from the overall-by-part chart. Lag band = 4–6 weeks (≈1–1.5-month freeze dwell). These June charts are Martins parts; Parks 666518 is not in this top-5 view.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="56" customHeight="true">
+      <c r="A36" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Original Tableau screenshots are not embedded here — the image files were not available to paste. Drop the two screenshots beside these tables if you want the visuals inline. Refresh monthly as new Tableau months arrive.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B6:C11 C15:C16 B21:B26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.05"/>
+        <cfvo type="num" val="0.1"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <mergeCells count="14">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A36:F36"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">

</xml_diff>

<commit_message>
ATM_Scrap tab: source-agnostic framing + native line chart
- Remove slaughterhouse attribution: ATM scrap is not divisible by SH (batch/lot
  numbers no longer tracked in Tableau); part number (666541/666506) is the only
  split. Updated subtitle, lag-table header/explainer, and notes.
- Fix line->part label: 666541 = the light-cyan series with the most data points
  (25%->0%); 666506 = the flatter near-zero series. Data mapping was already correct.
- Add a native Excel line chart (chart3) of the June scrap trend: 666541 vs 666506
  vs the 5% goal line, percent axis, value labels.
- Correct worksheet element order (mergeCells before conditionalFormatting).

Chart mirrors the workbook's existing chart structure; XML validated, workbook loads
cleanly. Defect Atlas photos and all other sheets unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014UGcEfvuC9NvQ5rauRTTbR
</commit_message>
<xml_diff>
--- a/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
+++ b/QC inspections suppliers/Pelvic_Blocks_Quality_062626.xlsx
@@ -3695,6 +3695,439 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:style val="2"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="en-US" sz="1400" b="1"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="1"/>
+              <a:t>ATM Scrap % Trend — June 2026 (666541 vs 666506)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ATM_Scrap_TableuData'!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>666541 Scrap %</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="4FB8CC"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="4FB8CC"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:numFmt formatCode="0.0%" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900"/>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ATM_Scrap_TableuData'!$A$6:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>5/25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6/1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6/8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6/15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6/22</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6/29</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ATM_Scrap_TableuData'!$B$6:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.063</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.074</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.032</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.032</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ATM_Scrap_TableuData'!$C$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>666506 Scrap %</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="9ECAE1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="9ECAE1"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:numFmt formatCode="0.0%" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900"/>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ATM_Scrap_TableuData'!$A$6:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>5/25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6/1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6/8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6/15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6/22</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6/29</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ATM_Scrap_TableuData'!$C$6:$C$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="1">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.014</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ATM_Scrap_TableuData'!$D$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Goal</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28800">
+              <a:solidFill>
+                <a:srgbClr val="9A9A9A"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:dLbls>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ATM_Scrap_TableuData'!$A$6:$A$11</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>5/25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6/1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6/8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6/15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6/22</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6/29</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ATM_Scrap_TableuData'!$D$6:$D$11</c:f>
+              <c:numCache>
+                <c:formatCode>0.0%</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.05</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="111111111"/>
+        <c:axId val="222222222"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="111111111"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="en-US" sz="1000" b="1"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1"/>
+                  <a:t>Week (ATM receipt)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="222222222"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="222222222"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr lang="en-US" sz="1000" b="1"/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1"/>
+                  <a:t>Scrap %</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="111111111"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="D9D9D9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -3995,6 +4428,41 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="ATM Scrap Trend Chart"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="7200000" cy="4000000"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -6332,10 +6800,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="true">
+    <row r="2" ht="72" customHeight="true">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Source: Tableau “Top 5 Part” scrap views, June 2026. ATM = receipt inspection AFTER freeze/thaw (product sits frozen ~1–1.5 months), so this month reflects SH harvest from roughly late-April to late-May. No batch/lot numbers in the ATM feed, so cross-stage links are by time-window + part only. Values read from the two charts.</t>
+          <t xml:space="preserve">Source: Tableau “Top 5 Part” scrap views, June 2026. ATM = receipt inspection AFTER freeze/thaw (product sits frozen ~1–1.5 months), so this month reflects SH harvest from roughly late-April to late-May. Batch/lot numbers are NOT tracked in the ATM feed, so scrap can only be split by part number (666541 / 666506) — not by slaughterhouse. Values read from the two charts.</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6968,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DV Tech Pelvic Block (F), intact — performance-goal part</t>
+          <t xml:space="preserve">Pelvic Block (F), intact — performance-goal part</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
@@ -6540,10 +7008,10 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="44" customHeight="true">
+    <row r="19" ht="56" customHeight="true">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Directional only: ATM is weekly, SH visits are sporadic, and there is no lot linkage. SH 666541 scrap below is from the Martins intact rows on the Slaughterhouse IQC tab for the matching harvest window.</t>
+          <t xml:space="preserve">Directional only: ATM is weekly, SH visits are sporadic, there is no lot linkage, and ATM can no longer be traced to a slaughterhouse. The SH scrap below is the female-intact scrap for the harvest window; Parks SH inspections only began 5/28, so these pre-June windows are Martins-dominated at the SH floor.</t>
         </is>
       </c>
     </row>
@@ -6565,7 +7033,7 @@
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">SH 666541 scrap (Martins)</t>
+          <t xml:space="preserve">SH female-intact scrap</t>
         </is>
       </c>
     </row>
@@ -6736,30 +7204,18 @@
     <row r="35" ht="56" customHeight="true">
       <c r="A35" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Line→part mapping (dark = 666541, light = 666506) inferred from the overall-by-part chart. Lag band = 4–6 weeks (≈1–1.5-month freeze dwell). These June charts are Martins parts; Parks 666518 is not in this top-5 view.</t>
+          <t xml:space="preserve">Line→part mapping: 666541 = the light-cyan line (the series with the most data points, 25% → 0%); 666506 = the flatter near-zero series. Lag band = 4–6 weeks (≈1–1.5-month freeze dwell).</t>
         </is>
       </c>
     </row>
     <row r="36" ht="56" customHeight="true">
       <c r="A36" s="20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Original Tableau screenshots are not embedded here — the image files were not available to paste. Drop the two screenshots beside these tables if you want the visuals inline. Refresh monthly as new Tableau months arrive.</t>
+          <t xml:space="preserve">ATM scrap can no longer be attributed to a slaughterhouse — batch/lot numbers are not tracked in Tableau, so a given ATM receipt can't be traced to Parks vs Martins; the part number (666541 intact, 666506 non-intact) is the only available split. Refresh monthly as new Tableau months arrive.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:C11 C15:C16 B21:B26">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.05"/>
-        <cfvo type="num" val="0.1"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <mergeCells count="14">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
@@ -6776,7 +7232,20 @@
     <mergeCell ref="A35:F35"/>
     <mergeCell ref="A36:F36"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6:C11 C15:C16 B21:B26">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.05"/>
+        <cfvo type="num" val="0.1"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>